<commit_message>
Update master Excel workbook and JSON test results for all 3 test case suites
</commit_message>
<xml_diff>
--- a/MICROSUN_OFFICIAL_TEST_REPORT.xlsx
+++ b/MICROSUN_OFFICIAL_TEST_REPORT.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="c:\Users\unite\OneDrive\Desktop\PDD\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F764E6A4-9573-4DEF-AE93-CE994F94A440}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DE8B6368-D09C-4501-904C-1DDC1DC5CDD9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="3675" yWindow="3675" windowWidth="21600" windowHeight="11835" firstSheet="5" activeTab="7" xr2:uid="{AFA13D81-8180-463B-BB9D-253AC2511CA3}"/>
   </bookViews>
@@ -4158,10 +4158,10 @@
     <t>Zero unhandled JavaScript runtime crashes detected (1 severe errors)</t>
   </si>
   <si>
-    <t>2026-08-20T11:54:11.176Z</t>
-  </si>
-  <si>
     <t>100.00% (24/24 Passed - ALL PASSED)</t>
+  </si>
+  <si>
+    <t>2026-08-20T12:34:45.366Z</t>
   </si>
 </sst>
 </file>
@@ -16515,7 +16515,7 @@
         <v>1364</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>1371</v>
+        <v>1372</v>
       </c>
     </row>
     <row r="5" spans="1:6" ht="16.5" x14ac:dyDescent="0.3">
@@ -16530,7 +16530,7 @@
         <v>1367</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>1372</v>
+        <v>1371</v>
       </c>
     </row>
     <row r="7" spans="1:6" ht="26.1" customHeight="1" x14ac:dyDescent="0.3">
@@ -16564,7 +16564,7 @@
         <v>132</v>
       </c>
       <c r="D8" s="26">
-        <v>578</v>
+        <v>392</v>
       </c>
       <c r="E8" s="27" t="s">
         <v>133</v>
@@ -16584,7 +16584,7 @@
         <v>136</v>
       </c>
       <c r="D9" s="30">
-        <v>198</v>
+        <v>85</v>
       </c>
       <c r="E9" s="27" t="s">
         <v>133</v>
@@ -16604,7 +16604,7 @@
         <v>139</v>
       </c>
       <c r="D10" s="26">
-        <v>955</v>
+        <v>857</v>
       </c>
       <c r="E10" s="27" t="s">
         <v>133</v>
@@ -16624,7 +16624,7 @@
         <v>143</v>
       </c>
       <c r="D11" s="30">
-        <v>208</v>
+        <v>71</v>
       </c>
       <c r="E11" s="27" t="s">
         <v>133</v>
@@ -16644,7 +16644,7 @@
         <v>147</v>
       </c>
       <c r="D12" s="26">
-        <v>450</v>
+        <v>260</v>
       </c>
       <c r="E12" s="27" t="s">
         <v>133</v>
@@ -16664,7 +16664,7 @@
         <v>150</v>
       </c>
       <c r="D13" s="30">
-        <v>103</v>
+        <v>53</v>
       </c>
       <c r="E13" s="27" t="s">
         <v>133</v>
@@ -16684,7 +16684,7 @@
         <v>154</v>
       </c>
       <c r="D14" s="26">
-        <v>61</v>
+        <v>35</v>
       </c>
       <c r="E14" s="27" t="s">
         <v>133</v>
@@ -16704,7 +16704,7 @@
         <v>158</v>
       </c>
       <c r="D15" s="30">
-        <v>579</v>
+        <v>447</v>
       </c>
       <c r="E15" s="27" t="s">
         <v>133</v>
@@ -16724,7 +16724,7 @@
         <v>161</v>
       </c>
       <c r="D16" s="26">
-        <v>554</v>
+        <v>534</v>
       </c>
       <c r="E16" s="27" t="s">
         <v>133</v>
@@ -16744,7 +16744,7 @@
         <v>164</v>
       </c>
       <c r="D17" s="30">
-        <v>560</v>
+        <v>539</v>
       </c>
       <c r="E17" s="27" t="s">
         <v>133</v>
@@ -16764,7 +16764,7 @@
         <v>167</v>
       </c>
       <c r="D18" s="26">
-        <v>645</v>
+        <v>591</v>
       </c>
       <c r="E18" s="27" t="s">
         <v>133</v>
@@ -16784,7 +16784,7 @@
         <v>171</v>
       </c>
       <c r="D19" s="30">
-        <v>2114</v>
+        <v>236</v>
       </c>
       <c r="E19" s="27" t="s">
         <v>133</v>
@@ -16804,7 +16804,7 @@
         <v>174</v>
       </c>
       <c r="D20" s="26">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="E20" s="27" t="s">
         <v>133</v>
@@ -16824,7 +16824,7 @@
         <v>178</v>
       </c>
       <c r="D21" s="30">
-        <v>683</v>
+        <v>489</v>
       </c>
       <c r="E21" s="27" t="s">
         <v>133</v>
@@ -16844,7 +16844,7 @@
         <v>181</v>
       </c>
       <c r="D22" s="26">
-        <v>19</v>
+        <v>12</v>
       </c>
       <c r="E22" s="27" t="s">
         <v>133</v>
@@ -16864,7 +16864,7 @@
         <v>185</v>
       </c>
       <c r="D23" s="30">
-        <v>584</v>
+        <v>427</v>
       </c>
       <c r="E23" s="27" t="s">
         <v>133</v>
@@ -16884,7 +16884,7 @@
         <v>188</v>
       </c>
       <c r="D24" s="26">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="E24" s="27" t="s">
         <v>133</v>
@@ -16904,7 +16904,7 @@
         <v>192</v>
       </c>
       <c r="D25" s="30">
-        <v>502</v>
+        <v>535</v>
       </c>
       <c r="E25" s="27" t="s">
         <v>133</v>
@@ -16924,7 +16924,7 @@
         <v>196</v>
       </c>
       <c r="D26" s="26">
-        <v>244</v>
+        <v>134</v>
       </c>
       <c r="E26" s="27" t="s">
         <v>133</v>
@@ -16944,7 +16944,7 @@
         <v>200</v>
       </c>
       <c r="D27" s="30">
-        <v>698</v>
+        <v>350</v>
       </c>
       <c r="E27" s="27" t="s">
         <v>133</v>
@@ -16964,7 +16964,7 @@
         <v>204</v>
       </c>
       <c r="D28" s="26">
-        <v>369</v>
+        <v>94</v>
       </c>
       <c r="E28" s="27" t="s">
         <v>133</v>
@@ -16984,7 +16984,7 @@
         <v>208</v>
       </c>
       <c r="D29" s="30">
-        <v>1638</v>
+        <v>1559</v>
       </c>
       <c r="E29" s="27" t="s">
         <v>133</v>
@@ -17004,7 +17004,7 @@
         <v>212</v>
       </c>
       <c r="D30" s="26">
-        <v>2594</v>
+        <v>1607</v>
       </c>
       <c r="E30" s="27" t="s">
         <v>133</v>
@@ -17024,7 +17024,7 @@
         <v>216</v>
       </c>
       <c r="D31" s="30">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E31" s="27" t="s">
         <v>133</v>

</xml_diff>